<commit_message>
chore: update input.xlsx example file to ExpenseType columns
</commit_message>
<xml_diff>
--- a/inst/app/www/examples/input.xlsx
+++ b/inst/app/www/examples/input.xlsx
@@ -4,7 +4,7 @@
   <workbookPr date1904="0"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="3" showHorizontalScroll="1" showVerticalScroll="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
     <sheet name="Expenses" sheetId="1" state="visible" r:id="rId1"/>
@@ -22,9 +22,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
-  <si>
-    <t>Type</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
+  <si>
+    <t>ExpenseType</t>
   </si>
   <si>
     <t>Reason</t>
@@ -310,9 +310,6 @@
   </si>
   <si>
     <t>Absent_Days</t>
-  </si>
-  <si>
-    <t>ExpenseType</t>
   </si>
   <si>
     <t>Percentage</t>
@@ -798,713 +795,713 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" ht="12.800000000000001">
-      <c r="A2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="2">
         <v>85.5</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" ht="12.800000000000001">
-      <c r="A3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
+      <c r="A3" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D3" s="2">
         <v>120</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" ht="12.800000000000001">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4" s="2">
         <v>45.75</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" ht="12.800000000000001">
-      <c r="A5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="2">
         <v>32.25</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" ht="12.800000000000001">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" s="2">
         <v>28.899999999999999</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" ht="12.800000000000001">
-      <c r="A7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="A7" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" s="2">
         <v>89</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" ht="12.800000000000001">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="2">
         <v>156.80000000000001</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" ht="12.800000000000001">
-      <c r="A9" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="A9" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" s="2">
         <v>92.150000000000006</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="10" ht="12.800000000000001">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="2">
         <v>18.5</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" ht="12.800000000000001">
-      <c r="A11" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="A11" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" s="2">
         <v>67.299999999999997</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="12" ht="12.800000000000001">
-      <c r="A12" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="1" t="s">
+      <c r="A12" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" s="2">
         <v>145.25</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" ht="12.800000000000001">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="D13" s="1">
+      <c r="D13" s="2">
         <v>55</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="14" ht="12.800000000000001">
-      <c r="A14" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="1" t="s">
+      <c r="A14" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="2">
         <v>24.800000000000001</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="15" ht="12.800000000000001">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D15" s="1">
+      <c r="D15" s="2">
         <v>89.400000000000006</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" ht="12.800000000000001">
-      <c r="A16" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="A16" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="2">
         <v>18.75</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="17" ht="12.800000000000001">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" s="2">
         <v>42.299999999999997</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="18" ht="12.800000000000001">
-      <c r="A18" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B18" s="1" t="s">
+      <c r="A18" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="1">
+      <c r="D18" s="2">
         <v>73.599999999999994</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="19" ht="12.800000000000001">
-      <c r="A19" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B19" s="1" t="s">
+      <c r="A19" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" s="2">
         <v>198.5</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="20" ht="12.800000000000001">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" s="2">
         <v>34.899999999999999</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="21" ht="12.800000000000001">
-      <c r="A21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="1" t="s">
+      <c r="A21" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D21" s="1">
+      <c r="D21" s="2">
         <v>12.449999999999999</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="22" ht="12.800000000000001">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D22" s="1">
+      <c r="D22" s="2">
         <v>96</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E22" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="23" ht="12.800000000000001">
-      <c r="A23" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B23" s="1" t="s">
+      <c r="A23" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D23" s="1">
+      <c r="D23" s="2">
         <v>112.3</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="E23" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="24" ht="12.800000000000001">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="D24" s="1">
+      <c r="D24" s="2">
         <v>78.200000000000003</v>
       </c>
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="25" ht="12.800000000000001">
-      <c r="A25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B25" s="1" t="s">
+      <c r="A25" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="1">
+      <c r="D25" s="2">
         <v>29.600000000000001</v>
       </c>
-      <c r="E25" s="1" t="s">
+      <c r="E25" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="26" ht="12.800000000000001">
-      <c r="A26" s="1" t="s">
+      <c r="A26" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="2">
         <v>125.40000000000001</v>
       </c>
-      <c r="E26" s="1" t="s">
+      <c r="E26" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="27" ht="12.800000000000001">
-      <c r="A27" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="A27" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D27" s="1">
+      <c r="D27" s="2">
         <v>22.149999999999999</v>
       </c>
-      <c r="E27" s="1" t="s">
+      <c r="E27" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="28" ht="12.800000000000001">
-      <c r="A28" s="1" t="s">
+      <c r="A28" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D28" s="1">
+      <c r="D28" s="2">
         <v>180</v>
       </c>
-      <c r="E28" s="1" t="s">
+      <c r="E28" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="29" ht="12.800000000000001">
-      <c r="A29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="A29" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C29" s="1" t="s">
+      <c r="C29" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" s="2">
         <v>15.800000000000001</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="E29" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="30" ht="12.800000000000001">
-      <c r="A30" s="1" t="s">
+      <c r="A30" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C30" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" s="2">
         <v>35.700000000000003</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="E30" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="31" ht="12.800000000000001">
-      <c r="A31" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="A31" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C31" s="1" t="s">
+      <c r="C31" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" s="2">
         <v>98.25</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E31" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="32" ht="12.800000000000001">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C32" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D32" s="2">
         <v>67.900000000000006</v>
       </c>
-      <c r="E32" s="1" t="s">
+      <c r="E32" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="33" ht="12.800000000000001">
-      <c r="A33" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B33" s="1" t="s">
+      <c r="A33" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C33" s="1" t="s">
+      <c r="C33" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D33" s="1">
+      <c r="D33" s="2">
         <v>41.200000000000003</v>
       </c>
-      <c r="E33" s="1" t="s">
+      <c r="E33" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="34" ht="12.800000000000001">
-      <c r="A34" s="1" t="s">
+      <c r="A34" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D34" s="1">
+      <c r="D34" s="2">
         <v>220</v>
       </c>
-      <c r="E34" s="1" t="s">
+      <c r="E34" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="35" ht="12.800000000000001">
-      <c r="A35" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B35" s="1" t="s">
+      <c r="A35" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C35" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D35" s="1">
+      <c r="D35" s="2">
         <v>19.300000000000001</v>
       </c>
-      <c r="E35" s="1" t="s">
+      <c r="E35" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="36" ht="12.800000000000001">
-      <c r="A36" s="1" t="s">
+      <c r="A36" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D36" s="1">
+      <c r="D36" s="2">
         <v>85.599999999999994</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="37" ht="12.800000000000001">
-      <c r="A37" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B37" s="1" t="s">
+      <c r="A37" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C37" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D37" s="1">
+      <c r="D37" s="2">
         <v>13.75</v>
       </c>
-      <c r="E37" s="1" t="s">
+      <c r="E37" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="38" ht="12.800000000000001">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="1" t="s">
+      <c r="C38" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="2">
         <v>156.80000000000001</v>
       </c>
-      <c r="E38" s="1" t="s">
+      <c r="E38" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="39" ht="12.800000000000001">
-      <c r="A39" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="A39" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C39" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D39" s="1">
+      <c r="D39" s="2">
         <v>87.400000000000006</v>
       </c>
-      <c r="E39" s="1" t="s">
+      <c r="E39" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="40" ht="12.800000000000001">
-      <c r="A40" s="1" t="s">
+      <c r="A40" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C40" s="1" t="s">
+      <c r="C40" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="D40" s="1">
+      <c r="D40" s="2">
         <v>72</v>
       </c>
-      <c r="E40" s="1" t="s">
+      <c r="E40" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="41" ht="12.800000000000001">
-      <c r="A41" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B41" s="1" t="s">
+      <c r="A41" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C41" s="1" t="s">
+      <c r="C41" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="1">
+      <c r="D41" s="2">
         <v>26.899999999999999</v>
       </c>
-      <c r="E41" s="1" t="s">
+      <c r="E41" s="2" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="42" ht="12.800000000000001">
-      <c r="A42" s="1" t="s">
+      <c r="A42" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="C42" s="1" t="s">
+      <c r="C42" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="D42" s="1">
+      <c r="D42" s="2">
         <v>95.5</v>
       </c>
-      <c r="E42" s="1" t="s">
+      <c r="E42" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -1618,41 +1615,41 @@
   </sheetPr>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.800000000000001"/>
   <cols>
-    <col customWidth="1" min="1" max="1" style="1" width="7.1600000000000001"/>
-    <col customWidth="1" min="2" max="2" style="1" width="7.3600000000000003"/>
-    <col customWidth="1" min="3" max="3" style="1" width="10.710000000000001"/>
+    <col customWidth="1" min="1" max="1" style="2" width="7.1600000000000001"/>
+    <col customWidth="1" min="2" max="2" style="2" width="7.3600000000000003"/>
+    <col customWidth="1" min="3" max="3" style="2" width="10.710000000000001"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.800000000000001">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>97</v>
-      </c>
     </row>
     <row r="2" ht="12.800000000000001">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="2">
         <v>0.20000000000000001</v>
       </c>
     </row>
     <row r="3" ht="12.800000000000001">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C3" s="2">
         <v>0.5</v>
       </c>
     </row>
@@ -1673,30 +1670,30 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.800000000000001"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" ht="12.800000000000001">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" ht="12.800000000000001">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" ht="12.800000000000001">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" ht="12.800000000000001">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" ht="12.800000000000001">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1720,28 +1717,28 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.800000000000001"/>
   <sheetData>
     <row r="1" ht="12.800000000000001">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" ht="12.800000000000001">
+      <c r="A2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" ht="12.800000000000001">
+      <c r="A3" s="2" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" ht="12.800000000000001">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" ht="12.800000000000001">
-      <c r="A3" s="1" t="s">
+    <row r="4" ht="12.800000000000001">
+      <c r="A4" s="2" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="4" ht="12.800000000000001">
-      <c r="A4" s="1" t="s">
+    <row r="5" ht="12.800000000000001">
+      <c r="A5" s="2" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="5" ht="12.800000000000001">
-      <c r="A5" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -1764,47 +1761,47 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.800000000000001"/>
   <sheetData>
     <row r="1" ht="12.800000000000001">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" ht="12.800000000000001">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" ht="12.800000000000001">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="4" ht="12.800000000000001">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" ht="12.800000000000001">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="6" ht="12.800000000000001">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="7" ht="12.800000000000001">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="8" ht="12.800000000000001">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="9" ht="12.800000000000001">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>30</v>
       </c>
     </row>

</xml_diff>